<commit_message>
added material for more chapters
</commit_message>
<xml_diff>
--- a/xl/stores.xlsx
+++ b/xl/stores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fz/Dev/python-for-excel/material/ch05/xl/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/dev/python-for-excel-2e/src/xl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51633E54-A744-9241-A7C6-F1255DF1AD26}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD9E05B9-DC0F-7E46-BC7A-F555B19D78BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="800" yWindow="460" windowWidth="29920" windowHeight="18740" xr2:uid="{DE96EA78-DEDB-0845-B68B-3B0A992487D5}"/>
+    <workbookView xWindow="2000" yWindow="-19600" windowWidth="29920" windowHeight="18740" xr2:uid="{DE96EA78-DEDB-0845-B68B-3B0A992487D5}"/>
   </bookViews>
   <sheets>
     <sheet name="2019" sheetId="1" r:id="rId1"/>
@@ -195,7 +195,32 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yy"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yy"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -208,10 +233,38 @@
 </styleSheet>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BA6BD420-57C9-C448-8DB2-9B2C6728773E}" name="Table2019" displayName="Table2019" ref="B2:F8" totalsRowShown="0">
+  <autoFilter ref="B2:F8" xr:uid="{BA6BD420-57C9-C448-8DB2-9B2C6728773E}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{31CB41E2-AD98-E143-84D1-8ADE399D2D8B}" name="Store"/>
+    <tableColumn id="2" xr3:uid="{DB50CD48-A30B-1140-AB98-DFC0D0FBC62F}" name="Employees"/>
+    <tableColumn id="3" xr3:uid="{790E60BC-6E15-EC49-B257-AFFD59BE6BC5}" name="Manager"/>
+    <tableColumn id="4" xr3:uid="{C0FE72FF-A1D1-A248-946D-64064499D6B4}" name="Since" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{347E6477-9CDB-7548-B792-35C05D46E30B}" name="Flagship"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{91E6FFBB-F90C-6F4D-95B0-F5A41664D027}" name="Table2020" displayName="Table2020" ref="B2:F8" totalsRowShown="0">
+  <autoFilter ref="B2:F8" xr:uid="{91E6FFBB-F90C-6F4D-95B0-F5A41664D027}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{14212866-0ED4-D84E-A612-5D6B198ECFF1}" name="Store"/>
+    <tableColumn id="2" xr3:uid="{32B48382-6992-8B48-9513-8AA928A240FB}" name="Employees" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{79BBA9EE-9A9D-F249-8ED7-73F50418909C}" name="Manager"/>
+    <tableColumn id="4" xr3:uid="{8DB0E394-F5F3-6B45-BAE4-15AA32269EF8}" name="Since" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{8BF9E652-88DF-1448-86E1-645C1E5ADD3A}" name="Flagship"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -249,7 +302,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -355,7 +408,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -497,7 +550,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -630,6 +683,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -758,6 +814,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>